<commit_message>
Papeles nuevos: graba las fechas del calendario DIAN como valores fijos (las formulas venian sin valor cacheado -> fecha limite salia vacia)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/PapelesTrabajo-EnBlanco.xlsx
+++ b/tests/fixtures/PapelesTrabajo-EnBlanco.xlsx
@@ -61,7 +61,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="20">
+  <numFmts count="21">
     <numFmt numFmtId="164" formatCode="#,##0_ ;\-#,##0\ "/>
     <numFmt numFmtId="165" formatCode="_-* #,##0\ _€_-;\-* #,##0\ _€_-;_-* &quot;-&quot;\ _€_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;\ #,##0;[Red]&quot;$&quot;\ \-#,##0"/>
@@ -82,6 +82,7 @@
     <numFmt numFmtId="181" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="182" formatCode="0_ "/>
     <numFmt numFmtId="183" formatCode="_ &quot;$&quot;\ * #,##0.00_ ;_ &quot;$&quot;\ * \-#,##0.00_ ;_ &quot;$&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="184" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="93">
     <font>
@@ -2287,7 +2288,7 @@
     <xf numFmtId="41" fontId="27" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1149">
+  <cellXfs count="1151">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -5439,6 +5440,8 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="32" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="2"/>
+    <xf numFmtId="184" fontId="31" fillId="23" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="184" fontId="31" fillId="26" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6166,9 +6169,6 @@
           <t xml:space="preserve">  🧾  Formulario 210 (autoritativo)</t>
         </is>
       </c>
-      <c r="C5" s="950" t="n"/>
-      <c r="D5" s="950" t="n"/>
-      <c r="E5" s="950" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="949" t="inlineStr">
@@ -6176,9 +6176,6 @@
           <t xml:space="preserve">  📄  Exógena 2025 — reportada por terceros</t>
         </is>
       </c>
-      <c r="C6" s="950" t="n"/>
-      <c r="D6" s="950" t="n"/>
-      <c r="E6" s="950" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="B7" s="951" t="inlineStr">
@@ -6193,9 +6190,6 @@
           <t xml:space="preserve">  💳  Deudas</t>
         </is>
       </c>
-      <c r="C8" s="950" t="n"/>
-      <c r="D8" s="950" t="n"/>
-      <c r="E8" s="950" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="B9" s="951" t="inlineStr">
@@ -6210,9 +6204,6 @@
           <t xml:space="preserve">  🏦  Rentas de capital</t>
         </is>
       </c>
-      <c r="C10" s="950" t="n"/>
-      <c r="D10" s="950" t="n"/>
-      <c r="E10" s="950" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="B11" s="951" t="inlineStr">
@@ -6227,9 +6218,6 @@
           <t xml:space="preserve">  👴  Cédula de pensiones</t>
         </is>
       </c>
-      <c r="C12" s="950" t="n"/>
-      <c r="D12" s="950" t="n"/>
-      <c r="E12" s="950" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="B13" s="951" t="inlineStr">
@@ -6244,9 +6232,6 @@
           <t xml:space="preserve">  🎯  Ganancias ocasionales</t>
         </is>
       </c>
-      <c r="C14" s="950" t="n"/>
-      <c r="D14" s="950" t="n"/>
-      <c r="E14" s="950" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="951" t="inlineStr">
@@ -6261,9 +6246,6 @@
           <t xml:space="preserve">  🧮  Retenciones en la fuente</t>
         </is>
       </c>
-      <c r="C16" s="950" t="n"/>
-      <c r="D16" s="950" t="n"/>
-      <c r="E16" s="950" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="B17" s="951" t="inlineStr">
@@ -6278,9 +6260,6 @@
           <t xml:space="preserve">  🎫  Descuentos tributarios</t>
         </is>
       </c>
-      <c r="C18" s="950" t="n"/>
-      <c r="D18" s="950" t="n"/>
-      <c r="E18" s="950" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="952" t="inlineStr">
@@ -6291,7 +6270,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B20:E20"/>
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B18:E18"/>
@@ -6305,6 +6283,7 @@
     <mergeCell ref="B11:E11"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B20:E20"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B10:E10"/>
     <mergeCell ref="B14:E14"/>
@@ -10883,7 +10862,7 @@
     <col width="19.83203125" customWidth="1" style="275" min="8" max="8"/>
     <col width="13.5" bestFit="1" customWidth="1" style="275" min="9" max="9"/>
     <col width="11" customWidth="1" style="275" min="10" max="15"/>
-    <col hidden="1" style="275" min="16" max="16"/>
+    <col hidden="1" width="13" customWidth="1" style="275" min="16" max="16"/>
     <col hidden="1" width="11" customWidth="1" style="275" min="17" max="16384"/>
   </cols>
   <sheetData>
@@ -12589,7 +12568,7 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="G67:G69"/>
     <mergeCell ref="G57:G59"/>
-    <mergeCell ref="H24:J30"/>
+    <mergeCell ref="G38:G44"/>
     <mergeCell ref="F54:F56"/>
     <mergeCell ref="G17:G23"/>
     <mergeCell ref="C31:C44"/>
@@ -12608,7 +12587,7 @@
     <mergeCell ref="B60:B62"/>
     <mergeCell ref="G3:G9"/>
     <mergeCell ref="B2:B30"/>
-    <mergeCell ref="G38:G44"/>
+    <mergeCell ref="H24:J30"/>
     <mergeCell ref="G10:G16"/>
   </mergeCells>
   <dataValidations count="1">
@@ -18129,9 +18108,8 @@
           <t>01</t>
         </is>
       </c>
-      <c r="C21" s="953">
-        <f>B8</f>
-        <v/>
+      <c r="C21" s="1149" t="n">
+        <v>46246</v>
       </c>
     </row>
     <row r="22">
@@ -18140,9 +18118,8 @@
           <t>02</t>
         </is>
       </c>
-      <c r="C22" s="953">
-        <f>C21</f>
-        <v/>
+      <c r="C22" s="1149" t="n">
+        <v>46246</v>
       </c>
     </row>
     <row r="23">
@@ -18151,9 +18128,8 @@
           <t>03</t>
         </is>
       </c>
-      <c r="C23" s="953">
-        <f>B9</f>
-        <v/>
+      <c r="C23" s="1149" t="n">
+        <v>46247</v>
       </c>
     </row>
     <row r="24">
@@ -18162,9 +18138,8 @@
           <t>04</t>
         </is>
       </c>
-      <c r="C24" s="953">
-        <f>C23</f>
-        <v/>
+      <c r="C24" s="1149" t="n">
+        <v>46247</v>
       </c>
     </row>
     <row r="25">
@@ -18173,9 +18148,8 @@
           <t>05</t>
         </is>
       </c>
-      <c r="C25" s="953">
-        <f>B10</f>
-        <v/>
+      <c r="C25" s="1149" t="n">
+        <v>46248</v>
       </c>
     </row>
     <row r="26">
@@ -18184,9 +18158,8 @@
           <t>06</t>
         </is>
       </c>
-      <c r="C26" s="953">
-        <f>C25</f>
-        <v/>
+      <c r="C26" s="1149" t="n">
+        <v>46248</v>
       </c>
     </row>
     <row r="27">
@@ -18195,9 +18168,8 @@
           <t>07</t>
         </is>
       </c>
-      <c r="C27" s="953">
-        <f>B11</f>
-        <v/>
+      <c r="C27" s="1149" t="n">
+        <v>46252</v>
       </c>
     </row>
     <row r="28">
@@ -18206,9 +18178,8 @@
           <t>08</t>
         </is>
       </c>
-      <c r="C28" s="953">
-        <f>C27</f>
-        <v/>
+      <c r="C28" s="1149" t="n">
+        <v>46252</v>
       </c>
     </row>
     <row r="29">
@@ -18217,9 +18188,8 @@
           <t>09</t>
         </is>
       </c>
-      <c r="C29" s="953">
-        <f>B12</f>
-        <v/>
+      <c r="C29" s="1149" t="n">
+        <v>46253</v>
       </c>
     </row>
     <row r="30">
@@ -18228,9 +18198,8 @@
           <t>10</t>
         </is>
       </c>
-      <c r="C30" s="953">
-        <f>C29</f>
-        <v/>
+      <c r="C30" s="1149" t="n">
+        <v>46253</v>
       </c>
     </row>
     <row r="31">
@@ -18239,9 +18208,8 @@
           <t>11</t>
         </is>
       </c>
-      <c r="C31" s="953">
-        <f>B13</f>
-        <v/>
+      <c r="C31" s="1149" t="n">
+        <v>46254</v>
       </c>
     </row>
     <row r="32">
@@ -18250,9 +18218,8 @@
           <t>12</t>
         </is>
       </c>
-      <c r="C32" s="953">
-        <f>C31</f>
-        <v/>
+      <c r="C32" s="1149" t="n">
+        <v>46254</v>
       </c>
     </row>
     <row r="33">
@@ -18261,9 +18228,8 @@
           <t>13</t>
         </is>
       </c>
-      <c r="C33" s="953">
-        <f>B14</f>
-        <v/>
+      <c r="C33" s="1149" t="n">
+        <v>46255</v>
       </c>
     </row>
     <row r="34">
@@ -18272,9 +18238,8 @@
           <t>14</t>
         </is>
       </c>
-      <c r="C34" s="953">
-        <f>C33</f>
-        <v/>
+      <c r="C34" s="1149" t="n">
+        <v>46255</v>
       </c>
     </row>
     <row r="35">
@@ -18283,9 +18248,8 @@
           <t>15</t>
         </is>
       </c>
-      <c r="C35" s="953">
-        <f>B15</f>
-        <v/>
+      <c r="C35" s="1149" t="n">
+        <v>46258</v>
       </c>
     </row>
     <row r="36">
@@ -18294,9 +18258,8 @@
           <t>16</t>
         </is>
       </c>
-      <c r="C36" s="953">
-        <f>C35</f>
-        <v/>
+      <c r="C36" s="1149" t="n">
+        <v>46258</v>
       </c>
     </row>
     <row r="37">
@@ -18305,9 +18268,8 @@
           <t>17</t>
         </is>
       </c>
-      <c r="C37" s="953">
-        <f>B16</f>
-        <v/>
+      <c r="C37" s="1149" t="n">
+        <v>46259</v>
       </c>
     </row>
     <row r="38">
@@ -18316,9 +18278,8 @@
           <t>18</t>
         </is>
       </c>
-      <c r="C38" s="953">
-        <f>C37</f>
-        <v/>
+      <c r="C38" s="1149" t="n">
+        <v>46259</v>
       </c>
     </row>
     <row r="39">
@@ -18327,9 +18288,8 @@
           <t>19</t>
         </is>
       </c>
-      <c r="C39" s="953">
-        <f>B17</f>
-        <v/>
+      <c r="C39" s="1149" t="n">
+        <v>46260</v>
       </c>
     </row>
     <row r="40">
@@ -18338,9 +18298,8 @@
           <t>20</t>
         </is>
       </c>
-      <c r="C40" s="953">
-        <f>C39</f>
-        <v/>
+      <c r="C40" s="1149" t="n">
+        <v>46260</v>
       </c>
     </row>
     <row r="41">
@@ -18349,9 +18308,8 @@
           <t>21</t>
         </is>
       </c>
-      <c r="C41" s="953">
-        <f>E8</f>
-        <v/>
+      <c r="C41" s="1149" t="n">
+        <v>46261</v>
       </c>
     </row>
     <row r="42">
@@ -18360,9 +18318,8 @@
           <t>22</t>
         </is>
       </c>
-      <c r="C42" s="953">
-        <f>C41</f>
-        <v/>
+      <c r="C42" s="1149" t="n">
+        <v>46261</v>
       </c>
     </row>
     <row r="43">
@@ -18371,9 +18328,8 @@
           <t>23</t>
         </is>
       </c>
-      <c r="C43" s="953">
-        <f>E9</f>
-        <v/>
+      <c r="C43" s="1149" t="n">
+        <v>46262</v>
       </c>
     </row>
     <row r="44">
@@ -18382,9 +18338,8 @@
           <t>24</t>
         </is>
       </c>
-      <c r="C44" s="953">
-        <f>C43</f>
-        <v/>
+      <c r="C44" s="1149" t="n">
+        <v>46262</v>
       </c>
     </row>
     <row r="45">
@@ -18393,9 +18348,8 @@
           <t>25</t>
         </is>
       </c>
-      <c r="C45" s="953">
-        <f>E10</f>
-        <v/>
+      <c r="C45" s="1149" t="n">
+        <v>46265</v>
       </c>
     </row>
     <row r="46">
@@ -18404,9 +18358,8 @@
           <t>26</t>
         </is>
       </c>
-      <c r="C46" s="953">
-        <f>C45</f>
-        <v/>
+      <c r="C46" s="1149" t="n">
+        <v>46265</v>
       </c>
     </row>
     <row r="47">
@@ -18415,9 +18368,8 @@
           <t>27</t>
         </is>
       </c>
-      <c r="C47" s="953">
-        <f>E11</f>
-        <v/>
+      <c r="C47" s="1149" t="n">
+        <v>46266</v>
       </c>
     </row>
     <row r="48">
@@ -18426,9 +18378,8 @@
           <t>28</t>
         </is>
       </c>
-      <c r="C48" s="953">
-        <f>C47</f>
-        <v/>
+      <c r="C48" s="1149" t="n">
+        <v>46266</v>
       </c>
     </row>
     <row r="49">
@@ -18437,9 +18388,8 @@
           <t>29</t>
         </is>
       </c>
-      <c r="C49" s="953">
-        <f>E12</f>
-        <v/>
+      <c r="C49" s="1149" t="n">
+        <v>46267</v>
       </c>
     </row>
     <row r="50">
@@ -18448,9 +18398,8 @@
           <t>30</t>
         </is>
       </c>
-      <c r="C50" s="953">
-        <f>C49</f>
-        <v/>
+      <c r="C50" s="1149" t="n">
+        <v>46267</v>
       </c>
     </row>
     <row r="51">
@@ -18459,9 +18408,8 @@
           <t>31</t>
         </is>
       </c>
-      <c r="C51" s="953">
-        <f>E13</f>
-        <v/>
+      <c r="C51" s="1149" t="n">
+        <v>46268</v>
       </c>
     </row>
     <row r="52">
@@ -18470,9 +18418,8 @@
           <t>32</t>
         </is>
       </c>
-      <c r="C52" s="953">
-        <f>C51</f>
-        <v/>
+      <c r="C52" s="1149" t="n">
+        <v>46268</v>
       </c>
     </row>
     <row r="53">
@@ -18481,9 +18428,8 @@
           <t>33</t>
         </is>
       </c>
-      <c r="C53" s="953">
-        <f>E14</f>
-        <v/>
+      <c r="C53" s="1149" t="n">
+        <v>46269</v>
       </c>
     </row>
     <row r="54">
@@ -18492,9 +18438,8 @@
           <t>34</t>
         </is>
       </c>
-      <c r="C54" s="953">
-        <f>C53</f>
-        <v/>
+      <c r="C54" s="1149" t="n">
+        <v>46269</v>
       </c>
     </row>
     <row r="55">
@@ -18503,9 +18448,8 @@
           <t>35</t>
         </is>
       </c>
-      <c r="C55" s="953">
-        <f>E15</f>
-        <v/>
+      <c r="C55" s="1149" t="n">
+        <v>46272</v>
       </c>
     </row>
     <row r="56">
@@ -18514,9 +18458,8 @@
           <t>36</t>
         </is>
       </c>
-      <c r="C56" s="953">
-        <f>C55</f>
-        <v/>
+      <c r="C56" s="1149" t="n">
+        <v>46272</v>
       </c>
     </row>
     <row r="57">
@@ -18525,9 +18468,8 @@
           <t>37</t>
         </is>
       </c>
-      <c r="C57" s="953">
-        <f>E16</f>
-        <v/>
+      <c r="C57" s="1149" t="n">
+        <v>46273</v>
       </c>
     </row>
     <row r="58">
@@ -18536,9 +18478,8 @@
           <t>38</t>
         </is>
       </c>
-      <c r="C58" s="953">
-        <f>C57</f>
-        <v/>
+      <c r="C58" s="1149" t="n">
+        <v>46273</v>
       </c>
     </row>
     <row r="59">
@@ -18547,9 +18488,8 @@
           <t>39</t>
         </is>
       </c>
-      <c r="C59" s="953">
-        <f>E17</f>
-        <v/>
+      <c r="C59" s="1149" t="n">
+        <v>46274</v>
       </c>
     </row>
     <row r="60">
@@ -18558,9 +18498,8 @@
           <t>40</t>
         </is>
       </c>
-      <c r="C60" s="953">
-        <f>C59</f>
-        <v/>
+      <c r="C60" s="1149" t="n">
+        <v>46274</v>
       </c>
     </row>
     <row r="61">
@@ -18569,9 +18508,8 @@
           <t>41</t>
         </is>
       </c>
-      <c r="C61" s="953">
-        <f>H8</f>
-        <v/>
+      <c r="C61" s="1149" t="n">
+        <v>46275</v>
       </c>
     </row>
     <row r="62">
@@ -18580,9 +18518,8 @@
           <t>42</t>
         </is>
       </c>
-      <c r="C62" s="953">
-        <f>C61</f>
-        <v/>
+      <c r="C62" s="1149" t="n">
+        <v>46275</v>
       </c>
     </row>
     <row r="63">
@@ -18591,9 +18528,8 @@
           <t>43</t>
         </is>
       </c>
-      <c r="C63" s="953">
-        <f>H9</f>
-        <v/>
+      <c r="C63" s="1149" t="n">
+        <v>46276</v>
       </c>
     </row>
     <row r="64">
@@ -18602,9 +18538,8 @@
           <t>44</t>
         </is>
       </c>
-      <c r="C64" s="953">
-        <f>C63</f>
-        <v/>
+      <c r="C64" s="1149" t="n">
+        <v>46276</v>
       </c>
     </row>
     <row r="65">
@@ -18613,9 +18548,8 @@
           <t>45</t>
         </is>
       </c>
-      <c r="C65" s="953">
-        <f>H10</f>
-        <v/>
+      <c r="C65" s="1149" t="n">
+        <v>46279</v>
       </c>
     </row>
     <row r="66">
@@ -18624,9 +18558,8 @@
           <t>46</t>
         </is>
       </c>
-      <c r="C66" s="953">
-        <f>C65</f>
-        <v/>
+      <c r="C66" s="1149" t="n">
+        <v>46279</v>
       </c>
     </row>
     <row r="67">
@@ -18635,9 +18568,8 @@
           <t>47</t>
         </is>
       </c>
-      <c r="C67" s="953">
-        <f>H11</f>
-        <v/>
+      <c r="C67" s="1149" t="n">
+        <v>46280</v>
       </c>
     </row>
     <row r="68">
@@ -18646,9 +18578,8 @@
           <t>48</t>
         </is>
       </c>
-      <c r="C68" s="953">
-        <f>C67</f>
-        <v/>
+      <c r="C68" s="1149" t="n">
+        <v>46280</v>
       </c>
     </row>
     <row r="69">
@@ -18657,9 +18588,8 @@
           <t>49</t>
         </is>
       </c>
-      <c r="C69" s="953">
-        <f>H12</f>
-        <v/>
+      <c r="C69" s="1149" t="n">
+        <v>46281</v>
       </c>
     </row>
     <row r="70">
@@ -18668,9 +18598,8 @@
           <t>50</t>
         </is>
       </c>
-      <c r="C70" s="953">
-        <f>C69</f>
-        <v/>
+      <c r="C70" s="1149" t="n">
+        <v>46281</v>
       </c>
     </row>
     <row r="71">
@@ -18679,9 +18608,8 @@
           <t>51</t>
         </is>
       </c>
-      <c r="C71" s="953">
-        <f>H13</f>
-        <v/>
+      <c r="C71" s="1149" t="n">
+        <v>46282</v>
       </c>
     </row>
     <row r="72">
@@ -18690,9 +18618,8 @@
           <t>52</t>
         </is>
       </c>
-      <c r="C72" s="953">
-        <f>C71</f>
-        <v/>
+      <c r="C72" s="1149" t="n">
+        <v>46282</v>
       </c>
     </row>
     <row r="73">
@@ -18701,9 +18628,8 @@
           <t>53</t>
         </is>
       </c>
-      <c r="C73" s="953">
-        <f>H14</f>
-        <v/>
+      <c r="C73" s="1149" t="n">
+        <v>46283</v>
       </c>
     </row>
     <row r="74">
@@ -18712,9 +18638,8 @@
           <t>54</t>
         </is>
       </c>
-      <c r="C74" s="953">
-        <f>C73</f>
-        <v/>
+      <c r="C74" s="1149" t="n">
+        <v>46283</v>
       </c>
     </row>
     <row r="75">
@@ -18723,9 +18648,8 @@
           <t>55</t>
         </is>
       </c>
-      <c r="C75" s="953">
-        <f>H15</f>
-        <v/>
+      <c r="C75" s="1149" t="n">
+        <v>46286</v>
       </c>
     </row>
     <row r="76">
@@ -18734,9 +18658,8 @@
           <t>56</t>
         </is>
       </c>
-      <c r="C76" s="953">
-        <f>C75</f>
-        <v/>
+      <c r="C76" s="1149" t="n">
+        <v>46286</v>
       </c>
     </row>
     <row r="77">
@@ -18745,9 +18668,8 @@
           <t>57</t>
         </is>
       </c>
-      <c r="C77" s="953">
-        <f>H16</f>
-        <v/>
+      <c r="C77" s="1149" t="n">
+        <v>46287</v>
       </c>
     </row>
     <row r="78">
@@ -18756,9 +18678,8 @@
           <t>58</t>
         </is>
       </c>
-      <c r="C78" s="953">
-        <f>C77</f>
-        <v/>
+      <c r="C78" s="1149" t="n">
+        <v>46287</v>
       </c>
     </row>
     <row r="79">
@@ -18767,9 +18688,8 @@
           <t>59</t>
         </is>
       </c>
-      <c r="C79" s="953">
-        <f>H17</f>
-        <v/>
+      <c r="C79" s="1149" t="n">
+        <v>46288</v>
       </c>
     </row>
     <row r="80">
@@ -18778,9 +18698,8 @@
           <t>60</t>
         </is>
       </c>
-      <c r="C80" s="955">
-        <f>C79</f>
-        <v/>
+      <c r="C80" s="1150" t="n">
+        <v>46288</v>
       </c>
     </row>
     <row r="81">
@@ -18789,9 +18708,8 @@
           <t>61</t>
         </is>
       </c>
-      <c r="C81" s="953">
-        <f>K8</f>
-        <v/>
+      <c r="C81" s="1149" t="n">
+        <v>46289</v>
       </c>
     </row>
     <row r="82">
@@ -18800,9 +18718,8 @@
           <t>62</t>
         </is>
       </c>
-      <c r="C82" s="953">
-        <f>C81</f>
-        <v/>
+      <c r="C82" s="1149" t="n">
+        <v>46289</v>
       </c>
     </row>
     <row r="83">
@@ -18811,9 +18728,8 @@
           <t>63</t>
         </is>
       </c>
-      <c r="C83" s="953">
-        <f>K9</f>
-        <v/>
+      <c r="C83" s="1149" t="n">
+        <v>46290</v>
       </c>
     </row>
     <row r="84">
@@ -18822,9 +18738,8 @@
           <t>64</t>
         </is>
       </c>
-      <c r="C84" s="953">
-        <f>C83</f>
-        <v/>
+      <c r="C84" s="1149" t="n">
+        <v>46290</v>
       </c>
     </row>
     <row r="85">
@@ -18833,9 +18748,8 @@
           <t>65</t>
         </is>
       </c>
-      <c r="C85" s="953">
-        <f>K10</f>
-        <v/>
+      <c r="C85" s="1149" t="n">
+        <v>46293</v>
       </c>
     </row>
     <row r="86">
@@ -18844,9 +18758,8 @@
           <t>66</t>
         </is>
       </c>
-      <c r="C86" s="953">
-        <f>C85</f>
-        <v/>
+      <c r="C86" s="1149" t="n">
+        <v>46293</v>
       </c>
     </row>
     <row r="87">
@@ -18855,9 +18768,8 @@
           <t>67</t>
         </is>
       </c>
-      <c r="C87" s="953">
-        <f>K11</f>
-        <v/>
+      <c r="C87" s="1149" t="n">
+        <v>46296</v>
       </c>
     </row>
     <row r="88">
@@ -18866,9 +18778,8 @@
           <t>68</t>
         </is>
       </c>
-      <c r="C88" s="953">
-        <f>C87</f>
-        <v/>
+      <c r="C88" s="1149" t="n">
+        <v>46296</v>
       </c>
     </row>
     <row r="89">
@@ -18877,9 +18788,8 @@
           <t>69</t>
         </is>
       </c>
-      <c r="C89" s="953">
-        <f>K12</f>
-        <v/>
+      <c r="C89" s="1149" t="n">
+        <v>46297</v>
       </c>
     </row>
     <row r="90">
@@ -18888,9 +18798,8 @@
           <t>70</t>
         </is>
       </c>
-      <c r="C90" s="953">
-        <f>C89</f>
-        <v/>
+      <c r="C90" s="1149" t="n">
+        <v>46297</v>
       </c>
     </row>
     <row r="91">
@@ -18899,9 +18808,8 @@
           <t>71</t>
         </is>
       </c>
-      <c r="C91" s="953">
-        <f>K13</f>
-        <v/>
+      <c r="C91" s="1149" t="n">
+        <v>46300</v>
       </c>
     </row>
     <row r="92">
@@ -18910,9 +18818,8 @@
           <t>72</t>
         </is>
       </c>
-      <c r="C92" s="953">
-        <f>C91</f>
-        <v/>
+      <c r="C92" s="1149" t="n">
+        <v>46300</v>
       </c>
     </row>
     <row r="93">
@@ -18921,9 +18828,8 @@
           <t>73</t>
         </is>
       </c>
-      <c r="C93" s="953">
-        <f>K14</f>
-        <v/>
+      <c r="C93" s="1149" t="n">
+        <v>46301</v>
       </c>
     </row>
     <row r="94">
@@ -18932,9 +18838,8 @@
           <t>74</t>
         </is>
       </c>
-      <c r="C94" s="953">
-        <f>C93</f>
-        <v/>
+      <c r="C94" s="1149" t="n">
+        <v>46301</v>
       </c>
     </row>
     <row r="95">
@@ -18943,9 +18848,8 @@
           <t>75</t>
         </is>
       </c>
-      <c r="C95" s="953">
-        <f>K15</f>
-        <v/>
+      <c r="C95" s="1149" t="n">
+        <v>46302</v>
       </c>
     </row>
     <row r="96">
@@ -18954,9 +18858,8 @@
           <t>76</t>
         </is>
       </c>
-      <c r="C96" s="953">
-        <f>C95</f>
-        <v/>
+      <c r="C96" s="1149" t="n">
+        <v>46302</v>
       </c>
     </row>
     <row r="97">
@@ -18965,9 +18868,8 @@
           <t>77</t>
         </is>
       </c>
-      <c r="C97" s="953">
-        <f>K16</f>
-        <v/>
+      <c r="C97" s="1149" t="n">
+        <v>46303</v>
       </c>
     </row>
     <row r="98">
@@ -18976,9 +18878,8 @@
           <t>78</t>
         </is>
       </c>
-      <c r="C98" s="953">
-        <f>C97</f>
-        <v/>
+      <c r="C98" s="1149" t="n">
+        <v>46303</v>
       </c>
     </row>
     <row r="99">
@@ -18987,9 +18888,8 @@
           <t>79</t>
         </is>
       </c>
-      <c r="C99" s="953">
-        <f>K17</f>
-        <v/>
+      <c r="C99" s="1149" t="n">
+        <v>46304</v>
       </c>
     </row>
     <row r="100">
@@ -18998,9 +18898,8 @@
           <t>80</t>
         </is>
       </c>
-      <c r="C100" s="953">
-        <f>C99</f>
-        <v/>
+      <c r="C100" s="1149" t="n">
+        <v>46304</v>
       </c>
     </row>
     <row r="101">
@@ -19009,9 +18908,8 @@
           <t>81</t>
         </is>
       </c>
-      <c r="C101" s="953">
-        <f>N8</f>
-        <v/>
+      <c r="C101" s="1149" t="n">
+        <v>46308</v>
       </c>
     </row>
     <row r="102">
@@ -19020,9 +18918,8 @@
           <t>82</t>
         </is>
       </c>
-      <c r="C102" s="953">
-        <f>C101</f>
-        <v/>
+      <c r="C102" s="1149" t="n">
+        <v>46308</v>
       </c>
     </row>
     <row r="103">
@@ -19031,9 +18928,8 @@
           <t>83</t>
         </is>
       </c>
-      <c r="C103" s="953">
-        <f>N9</f>
-        <v/>
+      <c r="C103" s="1149" t="n">
+        <v>46309</v>
       </c>
     </row>
     <row r="104">
@@ -19042,9 +18938,8 @@
           <t>84</t>
         </is>
       </c>
-      <c r="C104" s="953">
-        <f>C103</f>
-        <v/>
+      <c r="C104" s="1149" t="n">
+        <v>46309</v>
       </c>
     </row>
     <row r="105">
@@ -19053,9 +18948,8 @@
           <t>85</t>
         </is>
       </c>
-      <c r="C105" s="953">
-        <f>N10</f>
-        <v/>
+      <c r="C105" s="1149" t="n">
+        <v>46310</v>
       </c>
     </row>
     <row r="106">
@@ -19064,9 +18958,8 @@
           <t>86</t>
         </is>
       </c>
-      <c r="C106" s="953">
-        <f>C105</f>
-        <v/>
+      <c r="C106" s="1149" t="n">
+        <v>46310</v>
       </c>
     </row>
     <row r="107">
@@ -19075,9 +18968,8 @@
           <t>87</t>
         </is>
       </c>
-      <c r="C107" s="953">
-        <f>N11</f>
-        <v/>
+      <c r="C107" s="1149" t="n">
+        <v>46311</v>
       </c>
     </row>
     <row r="108">
@@ -19086,9 +18978,8 @@
           <t>88</t>
         </is>
       </c>
-      <c r="C108" s="953">
-        <f>C107</f>
-        <v/>
+      <c r="C108" s="1149" t="n">
+        <v>46311</v>
       </c>
     </row>
     <row r="109">
@@ -19097,9 +18988,8 @@
           <t>89</t>
         </is>
       </c>
-      <c r="C109" s="953">
-        <f>N12</f>
-        <v/>
+      <c r="C109" s="1149" t="n">
+        <v>46314</v>
       </c>
     </row>
     <row r="110">
@@ -19108,9 +18998,8 @@
           <t>90</t>
         </is>
       </c>
-      <c r="C110" s="953">
-        <f>C109</f>
-        <v/>
+      <c r="C110" s="1149" t="n">
+        <v>46314</v>
       </c>
     </row>
     <row r="111">
@@ -19119,9 +19008,8 @@
           <t>91</t>
         </is>
       </c>
-      <c r="C111" s="953">
-        <f>N13</f>
-        <v/>
+      <c r="C111" s="1149" t="n">
+        <v>46315</v>
       </c>
     </row>
     <row r="112">
@@ -19130,9 +19018,8 @@
           <t>92</t>
         </is>
       </c>
-      <c r="C112" s="953">
-        <f>C111</f>
-        <v/>
+      <c r="C112" s="1149" t="n">
+        <v>46315</v>
       </c>
     </row>
     <row r="113">
@@ -19141,9 +19028,8 @@
           <t>93</t>
         </is>
       </c>
-      <c r="C113" s="953">
-        <f>N14</f>
-        <v/>
+      <c r="C113" s="1149" t="n">
+        <v>46316</v>
       </c>
     </row>
     <row r="114">
@@ -19152,9 +19038,8 @@
           <t>94</t>
         </is>
       </c>
-      <c r="C114" s="953">
-        <f>C113</f>
-        <v/>
+      <c r="C114" s="1149" t="n">
+        <v>46316</v>
       </c>
     </row>
     <row r="115">
@@ -19163,9 +19048,8 @@
           <t>95</t>
         </is>
       </c>
-      <c r="C115" s="953">
-        <f>N15</f>
-        <v/>
+      <c r="C115" s="1149" t="n">
+        <v>46317</v>
       </c>
     </row>
     <row r="116">
@@ -19174,9 +19058,8 @@
           <t>96</t>
         </is>
       </c>
-      <c r="C116" s="953">
-        <f>C115</f>
-        <v/>
+      <c r="C116" s="1149" t="n">
+        <v>46317</v>
       </c>
     </row>
     <row r="117">
@@ -19185,9 +19068,8 @@
           <t>97</t>
         </is>
       </c>
-      <c r="C117" s="953">
-        <f>N16</f>
-        <v/>
+      <c r="C117" s="1149" t="n">
+        <v>46318</v>
       </c>
     </row>
     <row r="118">
@@ -19196,9 +19078,8 @@
           <t>98</t>
         </is>
       </c>
-      <c r="C118" s="953">
-        <f>C117</f>
-        <v/>
+      <c r="C118" s="1149" t="n">
+        <v>46318</v>
       </c>
     </row>
     <row r="119">
@@ -19207,9 +19088,8 @@
           <t>99</t>
         </is>
       </c>
-      <c r="C119" s="953">
-        <f>N17</f>
-        <v/>
+      <c r="C119" s="1149" t="n">
+        <v>46321</v>
       </c>
     </row>
     <row r="120">
@@ -19218,9 +19098,8 @@
           <t>00</t>
         </is>
       </c>
-      <c r="C120" s="953">
-        <f>C119</f>
-        <v/>
+      <c r="C120" s="1149" t="n">
+        <v>46321</v>
       </c>
     </row>
   </sheetData>
@@ -21105,7 +20984,7 @@
     <col width="19.5" customWidth="1" style="75" min="5" max="5"/>
     <col width="19" customWidth="1" style="72" min="6" max="6"/>
     <col width="11.5" customWidth="1" style="72" min="7" max="7"/>
-    <col hidden="1" style="72" min="8" max="8"/>
+    <col hidden="1" width="13" customWidth="1" style="72" min="8" max="8"/>
     <col hidden="1" width="11.5" customWidth="1" style="72" min="9" max="16384"/>
   </cols>
   <sheetData>
@@ -22296,7 +22175,7 @@
     <col hidden="1" width="10.83203125" customWidth="1" min="38" max="42"/>
     <col hidden="1" width="16.1640625" customWidth="1" min="43" max="43"/>
     <col hidden="1" width="11.1640625" customWidth="1" min="44" max="44"/>
-    <col hidden="1" min="45" max="48"/>
+    <col hidden="1" width="13" customWidth="1" min="45" max="48"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -26440,7 +26319,7 @@
     <col width="16" customWidth="1" style="69" min="9" max="9"/>
     <col width="31.6640625" customWidth="1" style="69" min="10" max="10"/>
     <col hidden="1" width="17.5" customWidth="1" style="69" min="11" max="13"/>
-    <col hidden="1" style="69" min="14" max="256"/>
+    <col hidden="1" width="13" customWidth="1" style="69" min="14" max="256"/>
     <col hidden="1" width="11.5" customWidth="1" style="69" min="257" max="16384"/>
   </cols>
   <sheetData>

</xml_diff>